<commit_message>
NT world met 2016-2019 en 2018-2019 split
</commit_message>
<xml_diff>
--- a/NorthernTrust/NT-KostenBepaling2020.xlsx
+++ b/NorthernTrust/NT-KostenBepaling2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GoogleDrive\Financieel\Aandelen\KeuzeWelkIndexFonds\PerFonds\NorthernTrust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79285619-07EF-4BA5-96C3-67C414ECE6EE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AE5F02-FFBB-4135-B81C-608494D05616}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -231,7 +231,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="101">
   <si>
     <t>Transaction costs and interest expenses are excluded from the calculation.</t>
   </si>
@@ -448,9 +448,6 @@
     <t>Alle kosten inc eventueel lek en drag</t>
   </si>
   <si>
-    <t>(over zelfde periode)</t>
-  </si>
-  <si>
     <t>TER wisselingen</t>
   </si>
   <si>
@@ -493,9 +490,6 @@
     <t>Kosten</t>
   </si>
   <si>
-    <t>TER en transactiekosten</t>
-  </si>
-  <si>
     <t>2016-2019</t>
   </si>
   <si>
@@ -518,6 +512,30 @@
   </si>
   <si>
     <t>todo</t>
+  </si>
+  <si>
+    <t>2018-2019</t>
+  </si>
+  <si>
+    <t>Op de 2017 factsheet adverteerde men wel met een 0.15% TER</t>
+  </si>
+  <si>
+    <t>TD 2018-2019</t>
+  </si>
+  <si>
+    <t>Huidige TER en transactiekosten</t>
+  </si>
+  <si>
+    <t>2016-2019 Alle kosten inc niet goed volgen index om onduidelijke redenen</t>
+  </si>
+  <si>
+    <t>2018-2019 Alle kosten inc niet goed volgen index om onduidelijke redenen</t>
+  </si>
+  <si>
+    <t>Feeder master structuur met cash drag?</t>
+  </si>
+  <si>
+    <t>Tracking Difference klopt niet door Swing pricing?</t>
   </si>
 </sst>
 </file>
@@ -644,7 +662,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -685,11 +703,12 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Komma" xfId="3" builtinId="3"/>
@@ -1056,15 +1075,15 @@
       <c r="B8" s="9"/>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="34"/>
+      <c r="B10" s="36"/>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="34"/>
+      <c r="B11" s="36"/>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
@@ -1162,7 +1181,7 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C2" s="30">
         <v>53732257.130000003</v>
@@ -1174,21 +1193,21 @@
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C4" s="30"/>
       <c r="G4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K4" t="s">
         <v>84</v>
-      </c>
-      <c r="K4" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C5" s="30">
         <v>41819772.990000002</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" s="7">
         <v>5.5E-2</v>
@@ -1202,23 +1221,23 @@
         <v>0.79995450026850634</v>
       </c>
       <c r="K5" s="4">
-        <f>World!C22</f>
-        <v>2.7774370256142822E-3</v>
+        <f>World!C27</f>
+        <v>2.7994627477833768E-3</v>
       </c>
       <c r="L5" s="6">
         <f>I5*K5</f>
-        <v>2.2218232478525197E-3</v>
+        <v>2.2394428234233507E-3</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C6" s="30">
         <v>5480574.1299999999</v>
       </c>
       <c r="F6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G6" s="7">
         <v>0.17699999999999999</v>
@@ -1242,13 +1261,13 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C7" s="30">
         <v>5789028.6699999999</v>
       </c>
       <c r="F7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G7" s="7">
         <v>7.1999999999999995E-2</v>
@@ -1272,13 +1291,13 @@
     </row>
     <row r="8" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C8" s="30">
         <v>642881.34999999963</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H8" s="32">
         <f>SUM(H5:H7)</f>
@@ -1286,12 +1305,12 @@
       </c>
       <c r="L8" s="6">
         <f>SUM(L5:L7)</f>
-        <v>2.9486176269170532E-3</v>
+        <v>2.9662372024878841E-3</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B9" s="29" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" s="31">
         <f>SUM(C5:C8)</f>
@@ -1304,12 +1323,12 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="G11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G12" s="7">
         <v>5.5E-2</v>
@@ -1321,7 +1340,7 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G13" s="7">
         <v>7.1999999999999995E-2</v>
@@ -1344,7 +1363,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J22"/>
+  <dimension ref="B2:J28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32.28515625" customWidth="1"/>
@@ -1395,7 +1414,7 @@
         <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -1415,6 +1434,9 @@
         <v>22294</v>
       </c>
       <c r="G5" s="3"/>
+      <c r="J5" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
@@ -1433,9 +1455,6 @@
         <v>2673847808</v>
       </c>
       <c r="G6" s="3"/>
-      <c r="J6" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -1460,6 +1479,9 @@
       <c r="G7" s="5"/>
       <c r="H7" s="6"/>
       <c r="I7" s="4"/>
+      <c r="J7" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -1483,9 +1505,6 @@
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="6"/>
-      <c r="J8" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
@@ -1513,7 +1532,7 @@
         <v>6.920931781713915E-5</v>
       </c>
       <c r="J9" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
@@ -1536,6 +1555,9 @@
       <c r="H10" s="7">
         <f t="shared" ref="H10" si="2">AVERAGE(C10:F10)</f>
         <v>8.25E-4</v>
+      </c>
+      <c r="J10" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
@@ -1546,9 +1568,6 @@
       <c r="F11" s="4"/>
       <c r="G11" s="5"/>
       <c r="H11" s="7"/>
-      <c r="J11" s="1" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
@@ -1568,8 +1587,8 @@
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
-      <c r="J12" t="s">
-        <v>66</v>
+      <c r="J12" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
@@ -1591,7 +1610,7 @@
       <c r="G13" s="5"/>
       <c r="H13" s="7"/>
       <c r="J13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
@@ -1620,7 +1639,7 @@
         <v>7.2553725221662438E-4</v>
       </c>
       <c r="J14" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1649,7 +1668,7 @@
         <v>7.3132805990583653E-4</v>
       </c>
       <c r="J15" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1659,8 +1678,11 @@
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J16" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>22</v>
       </c>
@@ -1669,14 +1691,17 @@
         <v>7.947465700337635E-4</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
       <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>62</v>
       </c>
@@ -1685,14 +1710,17 @@
         <v>2.0250000000000012E-3</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
       <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="J18" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>64</v>
       </c>
@@ -1700,13 +1728,15 @@
         <f>C18-C17</f>
         <v>1.2302534299662377E-3</v>
       </c>
-      <c r="D19" s="5"/>
+      <c r="D19" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="4"/>
       <c r="D20" s="5"/>
@@ -1715,33 +1745,102 @@
       <c r="G20" s="5"/>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="35">
-        <f>F10+AVERAGE(D9:F9)</f>
-        <v>1.5471835956480445E-3</v>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="7">
+        <f>AVERAGE(E14:F14)+AVERAGE(E9:F9)</f>
+        <v>1.2992112427753764E-3</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
       <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="4">
+        <f>'Tracking Difference'!O6/100</f>
+        <v>2.1000000000000085E-3</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="4">
+        <f>C22-C21</f>
+        <v>8.0078875722463215E-4</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="34">
+        <f>F10+H9</f>
+        <v>1.5692093178171392E-3</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C22" s="35">
-        <f>C21+C19</f>
-        <v>2.7774370256142822E-3</v>
-      </c>
-      <c r="D22" t="s">
-        <v>70</v>
+      <c r="C27" s="34">
+        <f>C25+C19</f>
+        <v>2.7994627477833768E-3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="34">
+        <f>C25+C23</f>
+        <v>2.3699980750417713E-3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1783,7 +1882,7 @@
         <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
@@ -1844,7 +1943,7 @@
       </c>
       <c r="G6" s="3"/>
       <c r="J6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
@@ -1896,7 +1995,7 @@
         <v>2.4500000000000004E-3</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2011,28 +2110,31 @@
       <c r="B15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="36">
+      <c r="C15" s="35">
         <f>H7+H12</f>
         <v>3.3249339540424843E-3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="35">
         <f>'Tracking Difference'!L15/100</f>
         <v>3.6750000000000016E-3</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>71</v>
+      <c r="D16" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="36">
+      <c r="C17" s="35">
         <f>C16-C15</f>
         <v>3.5006604595751731E-4</v>
       </c>
@@ -2040,13 +2142,13 @@
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
-      <c r="C18" s="36"/>
+      <c r="C18" s="35"/>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="34">
         <f>F8+AVERAGE(E7:F7)</f>
         <v>2.8678590481078306E-3</v>
       </c>
@@ -2058,7 +2160,7 @@
       <c r="B20" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="34">
         <f>C19+C17</f>
         <v>3.2179250940653479E-3</v>
       </c>
@@ -2127,7 +2229,7 @@
         <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -2228,7 +2330,7 @@
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H12" s="7"/>
     </row>
@@ -2262,7 +2364,7 @@
       <c r="B17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="36">
+      <c r="C17" s="35">
         <f>SUM(H7:H10)</f>
         <v>3.2090188294087553E-3</v>
       </c>
@@ -2524,13 +2626,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F528616F-4365-4E03-AA99-F5C2282C78C2}">
-  <dimension ref="B2:M16"/>
+  <dimension ref="B2:P16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="56.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="19">
         <v>2012</v>
@@ -2564,7 +2666,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" s="20" t="s">
         <v>56</v>
       </c>
@@ -2588,7 +2690,7 @@
       <c r="L3" s="18"/>
       <c r="M3" s="21"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" s="20" t="s">
         <v>57</v>
       </c>
@@ -2616,7 +2718,7 @@
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B5" s="20" t="s">
         <v>58</v>
       </c>
@@ -2640,7 +2742,7 @@
       <c r="L5" s="18"/>
       <c r="M5" s="21"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
         <v>59</v>
       </c>
@@ -2670,8 +2772,15 @@
         <v>0.20250000000000012</v>
       </c>
       <c r="M6" s="21"/>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="O6" s="37">
+        <f>AVERAGE(I6:J6)</f>
+        <v>0.21000000000000085</v>
+      </c>
+      <c r="P6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
         <v>60</v>
       </c>
@@ -2702,7 +2811,7 @@
         <v>0.42249999999999976</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="22"/>
       <c r="D11" s="23">
         <v>2013</v>
@@ -2733,7 +2842,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="24" t="s">
         <v>61</v>
       </c>
@@ -2756,7 +2865,7 @@
       <c r="L12" s="22"/>
       <c r="M12" s="25"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" s="24" t="s">
         <v>57</v>
       </c>
@@ -2783,7 +2892,7 @@
       <c r="L13" s="22"/>
       <c r="M13" s="25"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="24" t="s">
         <v>58</v>
       </c>
@@ -2806,7 +2915,7 @@
       <c r="L14" s="22"/>
       <c r="M14" s="25"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="24" t="s">
         <v>59</v>
       </c>
@@ -2836,7 +2945,7 @@
       </c>
       <c r="M15" s="25"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="24" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
NT EU en NA erbij, kleine fixes EM
</commit_message>
<xml_diff>
--- a/NorthernTrust/NT-KostenBepaling2020.xlsx
+++ b/NorthernTrust/NT-KostenBepaling2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GoogleDrive\Financieel\Aandelen\KeuzeWelkIndexFonds\PerFonds\NorthernTrust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A6493C-7BCC-4130-990A-B109A1FAEF8A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{557DAA49-9A10-4350-A9D9-B3BCC6AD50F1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,10 @@
     <sheet name="World" sheetId="1" r:id="rId3"/>
     <sheet name="Emerging" sheetId="5" r:id="rId4"/>
     <sheet name="SmallCaps" sheetId="6" r:id="rId5"/>
-    <sheet name="Northern Trust Master fondsen" sheetId="2" r:id="rId6"/>
-    <sheet name="Tracking Difference" sheetId="3" r:id="rId7"/>
+    <sheet name="NA" sheetId="10" r:id="rId6"/>
+    <sheet name="Europe" sheetId="11" r:id="rId7"/>
+    <sheet name="Northern Trust Master fondsen" sheetId="2" r:id="rId8"/>
+    <sheet name="Tracking Difference" sheetId="3" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,15 +43,42 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={5649945A-DA5B-4F3E-AD37-39E50C9D3093}</author>
     <author>tc={32D85BBB-ADB9-436B-A8F2-4522899AD645}</author>
+    <author>tc={E50F17E8-775B-49C3-97D7-B2F512BFCD2C}</author>
+    <author>tc={2BFD1DC0-1DA6-4E67-97B2-2CE5B3592E73}</author>
   </authors>
   <commentList>
-    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{32D85BBB-ADB9-436B-A8F2-4522899AD645}">
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{5649945A-DA5B-4F3E-AD37-39E50C9D3093}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    Uit statement of comprehensive income</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="1" shapeId="0" xr:uid="{32D85BBB-ADB9-436B-A8F2-4522899AD645}">
       <text>
         <t>[Opmerkingenthread]
 U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
 Opmerking:
     Uit 22. Portfolio Turnover Rate</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="2" shapeId="0" xr:uid="{E50F17E8-775B-49C3-97D7-B2F512BFCD2C}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    15. Ongoing Charges Figure</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="3" shapeId="0" xr:uid="{2BFD1DC0-1DA6-4E67-97B2-2CE5B3592E73}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    Uit statement of comprehensive income</t>
       </text>
     </comment>
   </commentList>
@@ -60,6 +89,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={BF773089-6A80-4D88-B46A-4941C8ADCD1E}</author>
+    <author>tc={B9734DE7-22D8-45D0-9EF6-06819DD1AEF6}</author>
   </authors>
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0" xr:uid="{BF773089-6A80-4D88-B46A-4941C8ADCD1E}">
@@ -70,6 +100,14 @@
     Uit 22. Portfolio Turnover Rate</t>
       </text>
     </comment>
+    <comment ref="B8" authorId="1" shapeId="0" xr:uid="{B9734DE7-22D8-45D0-9EF6-06819DD1AEF6}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    15. Ongoing Charges Figure</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -78,6 +116,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={4D1B1C4B-AE9C-4A11-936A-B15013E0FFB6}</author>
+    <author>tc={693A21C3-B684-4F83-8F88-788AD98B6C01}</author>
   </authors>
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0" xr:uid="{4D1B1C4B-AE9C-4A11-936A-B15013E0FFB6}">
@@ -88,6 +127,14 @@
     Uit 22. Portfolio Turnover Rate</t>
       </text>
     </comment>
+    <comment ref="B10" authorId="1" shapeId="0" xr:uid="{693A21C3-B684-4F83-8F88-788AD98B6C01}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    15. Ongoing Charges Figure</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -95,8 +142,64 @@
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={19782BDC-3516-452A-A148-93276D8F4BBB}</author>
+    <author>tc={5EB2339F-A6A8-4B4E-96BF-9F4706E8D87F}</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{19782BDC-3516-452A-A148-93276D8F4BBB}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    Uit 22. Portfolio Turnover Rate</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="1" shapeId="0" xr:uid="{5EB2339F-A6A8-4B4E-96BF-9F4706E8D87F}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    15. Ongoing Charges Figure</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={946B1519-DCF6-4AB0-8F53-062031767B1C}</author>
+    <author>tc={47B9A23D-4E39-4E7F-9EA4-13DC84F4C570}</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{946B1519-DCF6-4AB0-8F53-062031767B1C}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    Uit 22. Portfolio Turnover Rate</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="1" shapeId="0" xr:uid="{47B9A23D-4E39-4E7F-9EA4-13DC84F4C570}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    15. Ongoing Charges Figure</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
     <author>tc={BD318717-9F6E-4FE6-947A-CC33FA9CC4E4}</author>
     <author>tc={05F2B683-9025-489A-BD44-3439A44FEE41}</author>
+    <author>tc={25E7F969-6049-4206-AFF3-7E77554C6FC1}</author>
+    <author>tc={9B2ABA78-5EA9-4DFE-93AE-E8B1C32AF4D1}</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0" xr:uid="{BD318717-9F6E-4FE6-947A-CC33FA9CC4E4}">
@@ -117,17 +220,35 @@
 units" genomen uit "STATEMENT OF FINANCIAL POSITION"</t>
       </text>
     </comment>
+    <comment ref="B17" authorId="2" shapeId="0" xr:uid="{25E7F969-6049-4206-AFF3-7E77554C6FC1}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    "Net assets attributable to holders of redeemable participating
+units" genomen uit "STATEMENT OF FINANCIAL POSITION"</t>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="3" shapeId="0" xr:uid="{9B2ABA78-5EA9-4DFE-93AE-E8B1C32AF4D1}">
+      <text>
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
+    "Net assets attributable to holders of redeemable participating
+units" genomen uit "STATEMENT OF FINANCIAL POSITION"</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Gerben</author>
   </authors>
   <commentList>
-    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{434CD842-3C43-4334-B2E1-FAF0941512B8}">
+    <comment ref="J2" authorId="0" shapeId="0" xr:uid="{434CD842-3C43-4334-B2E1-FAF0941512B8}">
       <text>
         <r>
           <rPr>
@@ -151,7 +272,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M2" authorId="0" shapeId="0" xr:uid="{EE1FF351-82F3-401D-BF5F-E210234F658F}">
+    <comment ref="K2" authorId="0" shapeId="0" xr:uid="{EE1FF351-82F3-401D-BF5F-E210234F658F}">
       <text>
         <r>
           <rPr>
@@ -196,11 +317,12 @@
           </rPr>
           <t xml:space="preserve">
 Zelf moeten opzoeken in: https://www.msci.com/end-of-day-data-search
+Index suite: ESG Custom
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{491C301F-C58A-4556-8DFB-A3897F0CAD8E}">
+    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{491C301F-C58A-4556-8DFB-A3897F0CAD8E}">
       <text>
         <r>
           <rPr>
@@ -231,7 +353,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="115">
   <si>
     <t>Transaction costs and interest expenses are excluded from the calculation.</t>
   </si>
@@ -245,9 +367,6 @@
     <t>Northern Trust World Custom ESG Equity Index UCITS FGR Feeder Fund €</t>
   </si>
   <si>
-    <t>TER</t>
-  </si>
-  <si>
     <t>management</t>
   </si>
   <si>
@@ -309,9 +428,6 @@
   </si>
   <si>
     <t>06-2019 gestart. Feeder naar Northern Trust World Small Cap ESG Low Carbon Index Fund</t>
-  </si>
-  <si>
-    <t>Bij de world feeder worden er namelijk bijna geen kosten gemeld</t>
   </si>
   <si>
     <t>Aannames</t>
@@ -382,30 +498,18 @@
     <t>zou preciezer zijn, maar de bedragen zijn zo laag dat het waarschijnlijk geen verschil maakt</t>
   </si>
   <si>
-    <t>Operating costs</t>
-  </si>
-  <si>
     <t>Rente</t>
   </si>
   <si>
     <t>Allen maar 1x per jaar dividend uitkering, lopende dividenden worden wel meteen geinvesteerd?</t>
   </si>
   <si>
-    <t>% OC</t>
-  </si>
-  <si>
-    <t>% OC + Rente</t>
-  </si>
-  <si>
     <t>TD</t>
   </si>
   <si>
     <t>OPNI</t>
   </si>
   <si>
-    <t>Northern trust World Custom ESG Equity</t>
-  </si>
-  <si>
     <t>MSCI custom ESG (EUR) gross</t>
   </si>
   <si>
@@ -418,9 +522,6 @@
     <t>Vs net</t>
   </si>
   <si>
-    <t>NORTHERN TRUST EMERGING MARKETS CUSTOM ESG EQUITY</t>
-  </si>
-  <si>
     <t>Tracking difference</t>
   </si>
   <si>
@@ -439,9 +540,6 @@
     <t>Tax drag?</t>
   </si>
   <si>
-    <t>TER en transactie</t>
-  </si>
-  <si>
     <t>Schatting tracking diff toekomst</t>
   </si>
   <si>
@@ -493,9 +591,6 @@
     <t>2016-2019</t>
   </si>
   <si>
-    <t>De in rekening gebrachte TER lijkt soms lager als wat er in rekening gebracht had moeten worden</t>
-  </si>
-  <si>
     <t>Toch nog wat dividend lekkage?</t>
   </si>
   <si>
@@ -523,9 +618,6 @@
     <t>TD 2018-2019</t>
   </si>
   <si>
-    <t>Huidige TER en transactiekosten</t>
-  </si>
-  <si>
     <t>2016-2019 Alle kosten inc niet goed volgen index om onduidelijke redenen</t>
   </si>
   <si>
@@ -538,10 +630,76 @@
     <t>Tracking Difference klopt niet door Swing pricing?</t>
   </si>
   <si>
-    <t>Bruto netto index verschil</t>
-  </si>
-  <si>
-    <t>gemiddeld bruto netto index verschil</t>
+    <t>MSCI North America Custom ESG Index Net EUR</t>
+  </si>
+  <si>
+    <t>MSCI North America Custom ESG Index Gross EUR</t>
+  </si>
+  <si>
+    <t>Northern Trust North America Custom ESG Equity Index UCITS FGR Feeder Fund €</t>
+  </si>
+  <si>
+    <t>Northern Trust North America Custom ESG Equity Index UCITS FGR Feeder Fund</t>
+  </si>
+  <si>
+    <t>Northern Trust Emerging Markets Custom ESG Equity Index UCITS FGR Fund</t>
+  </si>
+  <si>
+    <t>Northern Trust World Custom ESG Equity Index UCITS FGR Feeder Fund</t>
+  </si>
+  <si>
+    <t>Northern Trust Europe Custom ESG Equity Index UCITS FGR Feeder Fund</t>
+  </si>
+  <si>
+    <t>MSCI Europe Custom ESG Index Net EUR</t>
+  </si>
+  <si>
+    <t>MSCI Europe Custom ESG Index Gross EUR</t>
+  </si>
+  <si>
+    <t>Northern Trust Europe Custom ESG Equity Index UCITS FGR Feeder Fund €</t>
+  </si>
+  <si>
+    <t>12-2015 gestart.  Feeder naar: Northern Trust North America Custom ESG Equity Index Fund (the "Master Fund")</t>
+  </si>
+  <si>
+    <t>Total operating exp - transaction</t>
+  </si>
+  <si>
+    <t>10-2015 gestart. Feeder naar:  Northern Trust Europe Custom ESG Equity Index Fund ("het master-fonds")</t>
+  </si>
+  <si>
+    <t>Northern Trust Europe ESG Equity Index Fund €</t>
+  </si>
+  <si>
+    <t>Northern Trust North America Custom ESG Equity Index Fund US$</t>
+  </si>
+  <si>
+    <t>TER gemeld</t>
+  </si>
+  <si>
+    <t>% TER in rekening gebracht</t>
+  </si>
+  <si>
+    <t>% TER in rekening gebracht + rente</t>
+  </si>
+  <si>
+    <t>Huidige TER en transactiekosten laatste jaren</t>
+  </si>
+  <si>
+    <t>Tussen de kosten benadering en tracking difference zit een flink gat</t>
+  </si>
+  <si>
+    <t>Bij de feeders worden er namelijk bijna geen transactiekosten gemeld</t>
+  </si>
+  <si>
+    <t>Tracking Difference kan vervuild zijn door de swing pricing, omdat swing pricing in de NAV zit</t>
+  </si>
+  <si>
+    <t>In emerging markets wat hogere transactiekosten</t>
+  </si>
+  <si>
+    <t>Transactiekosten ietwat aan de hoge kant voor europa</t>
   </si>
 </sst>
 </file>
@@ -555,9 +713,9 @@
     <numFmt numFmtId="165" formatCode="0.000%"/>
     <numFmt numFmtId="166" formatCode="0.0000%"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="176" formatCode="_ [$€-413]\ * #,##0_ ;_ [$€-413]\ * \-#,##0_ ;_ [$€-413]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -629,6 +787,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -674,7 +838,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -702,9 +866,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -717,13 +878,16 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Komma" xfId="3" builtinId="3"/>
@@ -1013,8 +1177,17 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B5" dT="2020-08-07T06:35:24.60" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{5649945A-DA5B-4F3E-AD37-39E50C9D3093}">
+    <text>Uit statement of comprehensive income</text>
+  </threadedComment>
   <threadedComment ref="B6" dT="2020-06-12T12:38:54.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{32D85BBB-ADB9-436B-A8F2-4522899AD645}">
     <text>Uit 22. Portfolio Turnover Rate</text>
+  </threadedComment>
+  <threadedComment ref="B10" dT="2020-08-07T06:59:33.92" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{E50F17E8-775B-49C3-97D7-B2F512BFCD2C}">
+    <text>15. Ongoing Charges Figure</text>
+  </threadedComment>
+  <threadedComment ref="B12" dT="2020-08-07T06:59:52.40" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{2BFD1DC0-1DA6-4E67-97B2-2CE5B3592E73}">
+    <text>Uit statement of comprehensive income</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -1024,6 +1197,9 @@
   <threadedComment ref="B6" dT="2020-06-12T12:38:54.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{BF773089-6A80-4D88-B46A-4941C8ADCD1E}">
     <text>Uit 22. Portfolio Turnover Rate</text>
   </threadedComment>
+  <threadedComment ref="B8" dT="2020-08-07T06:59:33.92" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{B9734DE7-22D8-45D0-9EF6-06819DD1AEF6}">
+    <text>15. Ongoing Charges Figure</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -1032,16 +1208,49 @@
   <threadedComment ref="B6" dT="2020-06-12T12:38:54.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{4D1B1C4B-AE9C-4A11-936A-B15013E0FFB6}">
     <text>Uit 22. Portfolio Turnover Rate</text>
   </threadedComment>
+  <threadedComment ref="B10" dT="2020-08-07T06:59:33.92" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{693A21C3-B684-4F83-8F88-788AD98B6C01}">
+    <text>15. Ongoing Charges Figure</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B6" dT="2020-06-12T12:38:54.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{19782BDC-3516-452A-A148-93276D8F4BBB}">
+    <text>Uit 22. Portfolio Turnover Rate</text>
+  </threadedComment>
+  <threadedComment ref="B10" dT="2020-08-07T06:59:33.92" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{5EB2339F-A6A8-4B4E-96BF-9F4706E8D87F}">
+    <text>15. Ongoing Charges Figure</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment5.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B6" dT="2020-06-12T12:38:54.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{946B1519-DCF6-4AB0-8F53-062031767B1C}">
+    <text>Uit 22. Portfolio Turnover Rate</text>
+  </threadedComment>
+  <threadedComment ref="B10" dT="2020-08-07T06:59:33.92" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{47B9A23D-4E39-4E7F-9EA4-13DC84F4C570}">
+    <text>15. Ongoing Charges Figure</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment6.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B5" dT="2020-06-17T17:48:02.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{BD318717-9F6E-4FE6-947A-CC33FA9CC4E4}">
     <text>"Net assets attributable to holders of redeemable participating
 units" genomen uit "STATEMENT OF FINANCIAL POSITION"</text>
   </threadedComment>
   <threadedComment ref="B11" dT="2020-06-17T17:48:02.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{05F2B683-9025-489A-BD44-3439A44FEE41}">
+    <text>"Net assets attributable to holders of redeemable participating
+units" genomen uit "STATEMENT OF FINANCIAL POSITION"</text>
+  </threadedComment>
+  <threadedComment ref="B17" dT="2020-06-17T17:48:02.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{25E7F969-6049-4206-AFF3-7E77554C6FC1}">
+    <text>"Net assets attributable to holders of redeemable participating
+units" genomen uit "STATEMENT OF FINANCIAL POSITION"</text>
+  </threadedComment>
+  <threadedComment ref="B23" dT="2020-06-17T17:48:02.75" personId="{A4396B54-26D6-4DB8-90A1-70B73ABD3ACC}" id="{9B2ABA78-5EA9-4DFE-93AE-E8B1C32AF4D1}">
     <text>"Net assets attributable to holders of redeemable participating
 units" genomen uit "STATEMENT OF FINANCIAL POSITION"</text>
   </threadedComment>
@@ -1058,31 +1267,31 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="26" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="26" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1090,32 +1299,32 @@
       <c r="B8" s="9"/>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="40" t="s">
-        <v>36</v>
+      <c r="B9" s="37" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="40"/>
+      <c r="B10" s="37"/>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="40"/>
+      <c r="B11" s="37"/>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="16"/>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
@@ -1123,22 +1332,22 @@
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>26</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
@@ -1146,7 +1355,7 @@
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
@@ -1154,24 +1363,26 @@
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30" s="2"/>
+      <c r="B30" s="2" t="s">
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1196,107 +1407,107 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="29">
+        <v>65</v>
+      </c>
+      <c r="C2" s="28">
         <v>53732257.130000003</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C3" s="29"/>
+      <c r="C3" s="28"/>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C4" s="29"/>
+      <c r="C4" s="28"/>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="K4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="29">
+        <v>66</v>
+      </c>
+      <c r="C5" s="28">
         <v>41819772.990000002</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G5" s="7">
         <v>5.5E-2</v>
       </c>
-      <c r="H5" s="31">
+      <c r="H5" s="30">
         <f>C5*(100%-G5)</f>
         <v>39519685.475550003</v>
       </c>
-      <c r="I5" s="32">
+      <c r="I5" s="31">
         <f>H5/$H$8</f>
         <v>0.79995450026850634</v>
       </c>
       <c r="K5" s="4">
-        <f>World!C27</f>
-        <v>2.7994627477833768E-3</v>
+        <f>World!C28</f>
+        <v>2.7658110617113322E-3</v>
       </c>
       <c r="L5" s="6">
         <f>I5*K5</f>
-        <v>2.2394428234233507E-3</v>
+        <v>2.2125230057083957E-3</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="29">
+        <v>67</v>
+      </c>
+      <c r="C6" s="28">
         <v>5480574.1299999999</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G6" s="7">
         <v>0.17699999999999999</v>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="30">
         <f>C6*(100%-G6)</f>
         <v>4510512.50899</v>
       </c>
-      <c r="I6" s="32">
+      <c r="I6" s="31">
         <f t="shared" ref="I6:I7" si="0">H6/$H$8</f>
         <v>9.1301454874084517E-2</v>
       </c>
       <c r="K6" s="4">
-        <f>Emerging!C20</f>
-        <v>3.2179250940653479E-3</v>
+        <f>Emerging!C21</f>
+        <v>3.3884138967802441E-3</v>
       </c>
       <c r="L6" s="6">
         <f t="shared" ref="L6:L7" si="1">I6*K6</f>
-        <v>2.9380124276399153E-4</v>
+        <v>3.0936711849160233E-4</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="29">
+        <v>68</v>
+      </c>
+      <c r="C7" s="28">
         <v>5789028.6699999999</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="G7" s="7">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="30">
         <f>C7*(100%-G7)</f>
         <v>5372218.6057600006</v>
       </c>
-      <c r="I7" s="32">
+      <c r="I7" s="31">
         <f t="shared" si="0"/>
         <v>0.10874404485740921</v>
       </c>
       <c r="K7" s="4">
-        <f>SmallCaps!C20</f>
+        <f>SmallCaps!C21</f>
         <v>3.9817641220565667E-3</v>
       </c>
       <c r="L7" s="6">
@@ -1306,67 +1517,67 @@
     </row>
     <row r="8" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="29">
+        <v>69</v>
+      </c>
+      <c r="C8" s="28">
         <v>642881.34999999963</v>
       </c>
       <c r="D8" t="s">
-        <v>78</v>
-      </c>
-      <c r="H8" s="31">
+        <v>70</v>
+      </c>
+      <c r="H8" s="30">
         <f>SUM(H5:H7)</f>
         <v>49402416.590300001</v>
       </c>
       <c r="L8" s="6">
         <f>SUM(L5:L7)</f>
-        <v>2.9662372024878841E-3</v>
+        <v>2.9548832605005401E-3</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="30">
+      <c r="B9" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="29">
         <f>SUM(C5:C8)</f>
         <v>53732257.140000008</v>
       </c>
-      <c r="H9" s="26">
+      <c r="H9" s="25">
         <f>SUM(H5:H7)/C2</f>
         <v>0.91941822713264454</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="G11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G12" s="7">
         <v>5.5E-2</v>
       </c>
-      <c r="H12" s="31">
+      <c r="H12" s="30">
         <f>C5*(100%-G12)</f>
         <v>39519685.475550003</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="G13" s="7">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="H13" s="31">
+      <c r="H13" s="30">
         <f>C7*(100%-G13)</f>
         <v>5372218.6057600006</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="H16" s="26">
+      <c r="H16" s="25">
         <f>SUM(H12:H13)/C2</f>
         <v>0.83547400535768268</v>
       </c>
@@ -1378,7 +1589,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J28"/>
+  <dimension ref="B2:J29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32.28515625" customWidth="1"/>
@@ -1400,15 +1611,15 @@
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="J2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
@@ -1426,10 +1637,10 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -1450,12 +1661,12 @@
       </c>
       <c r="G5" s="3"/>
       <c r="J5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="13">
         <v>607319449</v>
@@ -1473,7 +1684,7 @@
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="5">
         <f>C5/C6</f>
@@ -1495,12 +1706,12 @@
       <c r="H7" s="6"/>
       <c r="I7" s="4"/>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="5">
         <f>'Northern Trust Master fondsen'!D6</f>
@@ -1523,7 +1734,7 @@
     </row>
     <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C9" s="5">
         <f>SUM(C7:C8)</f>
@@ -1547,12 +1758,12 @@
         <v>6.920931781713915E-5</v>
       </c>
       <c r="J9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="C10" s="4">
         <v>2.9999999999999997E-4</v>
@@ -1572,7 +1783,7 @@
         <v>8.25E-4</v>
       </c>
       <c r="J10" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
@@ -1586,29 +1797,32 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="C12" s="17">
-        <v>72708</v>
+        <v>159521</v>
       </c>
       <c r="D12" s="17">
+        <f>323257-D5</f>
         <v>323257</v>
       </c>
       <c r="E12" s="17">
+        <f>2280765-E5</f>
         <v>2280765</v>
       </c>
       <c r="F12" s="17">
-        <v>3265001</v>
+        <f>3265001-F5</f>
+        <v>3242707</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="7"/>
       <c r="J12" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C13" s="17">
         <v>1794</v>
@@ -1625,16 +1839,16 @@
       <c r="G13" s="5"/>
       <c r="H13" s="7"/>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="C14" s="4">
         <f>C12/C6</f>
-        <v>1.1971953165623055E-4</v>
+        <v>2.6266407285764366E-4</v>
       </c>
       <c r="D14" s="4">
         <f t="shared" ref="D14:F14" si="3">D12/D6</f>
@@ -1646,24 +1860,24 @@
       </c>
       <c r="F14" s="4">
         <f t="shared" si="3"/>
-        <v>1.2210870754241522E-3</v>
+        <v>1.212749278510918E-3</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="7">
         <f>AVERAGE(C14:F14)</f>
-        <v>7.2553725221662438E-4</v>
+        <v>7.5918893828866914E-4</v>
       </c>
       <c r="J14" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="C15" s="4">
         <f>(C12+C13)/C6</f>
-        <v>1.2267349600391276E-4</v>
+        <v>2.6561803720532586E-4</v>
       </c>
       <c r="D15" s="4">
         <f t="shared" ref="D15:F15" si="4">(D12+D13)/D6</f>
@@ -1675,102 +1889,95 @@
       </c>
       <c r="F15" s="4">
         <f t="shared" si="4"/>
-        <v>1.2329654627822408E-3</v>
+        <v>1.2246276658690067E-3</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="7">
         <f>AVERAGE(C15:F15)</f>
-        <v>7.3132805990583653E-4</v>
+        <v>7.649797459778813E-4</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="6"/>
-      <c r="J16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="7">
-        <f>H9+H14</f>
-        <v>7.947465700337635E-4</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>85</v>
-      </c>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
       <c r="H17" s="6"/>
       <c r="J17" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" s="4">
-        <f>'Tracking Difference'!L6/100</f>
-        <v>2.0250000000000012E-3</v>
+        <v>21</v>
+      </c>
+      <c r="C18" s="7">
+        <f>H9+H14</f>
+        <v>8.2839825610580827E-4</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
       <c r="H18" s="6"/>
       <c r="J18" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="C19" s="4">
-        <f>C18-C17</f>
-        <v>1.2302534299662377E-3</v>
+        <f>'Tracking Difference'!J7/100</f>
+        <v>2.0250000000000012E-3</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
       <c r="H19" s="6"/>
+      <c r="J19" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="5"/>
+      <c r="B20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="4">
+        <f>C19-C18</f>
+        <v>1.196601743894193E-3</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>77</v>
+      </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
       <c r="H20" s="6"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="7">
-        <f>AVERAGE(E14:F14)+AVERAGE(E9:F9)</f>
-        <v>1.2992112427753764E-3</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>93</v>
-      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
@@ -1778,14 +1985,14 @@
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C22" s="4">
-        <f>'Tracking Difference'!O6/100</f>
-        <v>2.1000000000000085E-3</v>
+        <v>21</v>
+      </c>
+      <c r="C22" s="7">
+        <f>AVERAGE(E14:F14)+AVERAGE(E9:F9)</f>
+        <v>1.2950423443187594E-3</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
@@ -1794,14 +2001,14 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="C23" s="4">
-        <f>C22-C21</f>
-        <v>8.0078875722463215E-4</v>
+        <f>'Tracking Difference'!M7/100</f>
+        <v>2.1000000000000085E-3</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
@@ -1809,53 +2016,69 @@
       <c r="H23" s="6"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="5"/>
+      <c r="B24" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="4">
+        <f>C23-C22</f>
+        <v>8.0495765568124912E-4</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
       <c r="H24" s="6"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="33">
-        <f>F10+H9</f>
-        <v>1.5692093178171392E-3</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>96</v>
-      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
       <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C27" s="33">
-        <f>C25+C19</f>
-        <v>2.7994627477833768E-3</v>
-      </c>
-      <c r="D27" t="s">
-        <v>97</v>
-      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="32">
+        <f>F10+H9</f>
+        <v>1.5692093178171392E-3</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C28" s="33">
-        <f>C25+C23</f>
-        <v>2.3699980750417713E-3</v>
+        <v>61</v>
+      </c>
+      <c r="C28" s="32">
+        <f>C26+C20</f>
+        <v>2.7658110617113322E-3</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="32">
+        <f>C26+C24</f>
+        <v>2.3741669734983883E-3</v>
+      </c>
+      <c r="D29" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +2090,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F5B4C98-CE28-4015-A5EF-F840D4E9DB1C}">
-  <dimension ref="B2:J20"/>
+  <dimension ref="B2:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="33.28515625" customWidth="1"/>
@@ -1889,15 +2112,15 @@
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="J2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J3" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
@@ -1916,10 +2139,10 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -1942,10 +2165,10 @@
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3">
-        <v>41072828</v>
+        <v>72832569</v>
       </c>
       <c r="D6" s="3">
         <v>280855994</v>
@@ -1958,16 +2181,16 @@
       </c>
       <c r="G6" s="3"/>
       <c r="J6" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="4">
         <f>C5/C6</f>
-        <v>1.177079893305618E-3</v>
+        <v>6.6379643974936542E-4</v>
       </c>
       <c r="D7" s="4">
         <f t="shared" ref="D7:F7" si="0">D5/D6</f>
@@ -1984,13 +2207,13 @@
       <c r="G7" s="5"/>
       <c r="H7" s="7">
         <f>AVERAGE(C7:F7)</f>
-        <v>7.2449119660608022E-4</v>
+        <v>5.9617033321701716E-4</v>
       </c>
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="C8" s="7">
         <v>2.8E-3</v>
@@ -2010,7 +2233,7 @@
         <v>2.4500000000000004E-3</v>
       </c>
       <c r="J8" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2024,29 +2247,36 @@
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="C10" s="3">
-        <v>51166</v>
+        <f>252128-C5</f>
+        <v>203782</v>
       </c>
       <c r="D10" s="3">
-        <v>842623</v>
+        <f>842623-D5</f>
+        <v>565933</v>
       </c>
       <c r="E10" s="3">
-        <v>2541872</v>
+        <f>2541872-E5</f>
+        <v>2307298</v>
       </c>
       <c r="F10" s="3">
-        <v>4524697</v>
+        <f>4524697-F5</f>
+        <v>3852014</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="7"/>
+      <c r="J10" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C11" s="3">
-        <v>885</v>
+        <v>0</v>
       </c>
       <c r="D11" s="3">
         <v>35778</v>
@@ -2062,130 +2292,139 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="C12" s="4">
         <f>C10/C6</f>
-        <v>1.2457384234657522E-3</v>
+        <v>2.7979515592811231E-3</v>
       </c>
       <c r="D12" s="4">
         <f>D10/D6</f>
-        <v>3.0001958939854423E-3</v>
+        <v>2.0150290970824001E-3</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" ref="E12:F12" si="1">E10/E6</f>
-        <v>3.1828391782400471E-3</v>
+        <v>2.8891141923255395E-3</v>
       </c>
       <c r="F12" s="4">
         <f t="shared" si="1"/>
-        <v>2.9729975340543747E-3</v>
+        <v>2.5310044237532212E-3</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="7">
         <f>AVERAGE(C12:F12)</f>
-        <v>2.6004427574364041E-3</v>
+        <v>2.5582748181105712E-3</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="C13" s="4">
         <f>(C10+C11)/C6</f>
-        <v>1.267285515377709E-3</v>
+        <v>2.7979515592811231E-3</v>
       </c>
       <c r="D13" s="4">
         <f t="shared" ref="D13:F13" si="2">(D10+D11)/D6</f>
-        <v>3.1275850213828798E-3</v>
+        <v>2.142418224479838E-3</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="2"/>
-        <v>3.2020047917965685E-3</v>
+        <v>2.9082798058820609E-3</v>
       </c>
       <c r="F13" s="4">
         <f t="shared" si="2"/>
-        <v>2.9806693669323816E-3</v>
+        <v>2.5386762566312281E-3</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="7">
         <f>AVERAGE(C13:F13)</f>
-        <v>2.6443861738723847E-3</v>
+        <v>2.5968314615685624E-3</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="34">
-        <f>H7+H12</f>
-        <v>3.3249339540424843E-3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>85</v>
-      </c>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="2"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="34">
-        <f>'Tracking Difference'!L15/100</f>
-        <v>3.6750000000000016E-3</v>
+        <v>21</v>
+      </c>
+      <c r="C16" s="33">
+        <f>H7+H12</f>
+        <v>3.1544451513275881E-3</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="34">
-        <f>C16-C15</f>
-        <v>3.5006604595751731E-4</v>
-      </c>
-      <c r="D17" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="C17" s="33">
+        <f>'Tracking Difference'!J14/100</f>
+        <v>3.6750000000000016E-3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="34"/>
+      <c r="B18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="33">
+        <f>C17-C16</f>
+        <v>5.2055484867241349E-4</v>
+      </c>
+      <c r="D18" s="5"/>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="33">
+      <c r="B19" s="2"/>
+      <c r="C19" s="33"/>
+    </row>
+    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="32">
         <f>F8+AVERAGE(E7:F7)</f>
         <v>2.8678590481078306E-3</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" s="33">
-        <f>C19+C17</f>
-        <v>3.2179250940653479E-3</v>
-      </c>
-      <c r="D20" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="6"/>
+      <c r="D20" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="32">
+        <f>C20+C18</f>
+        <v>3.3884138967802441E-3</v>
+      </c>
+      <c r="D21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2196,10 +2435,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9123B064-D487-424B-955E-970CD2CDF897}">
-  <dimension ref="B2:J21"/>
+  <dimension ref="B2:J22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="31" customWidth="1"/>
     <col min="3" max="6" width="17.7109375" customWidth="1"/>
     <col min="7" max="7" width="6.140625" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
@@ -2209,7 +2448,7 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
@@ -2218,12 +2457,12 @@
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="J2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
@@ -2241,10 +2480,10 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
@@ -2261,7 +2500,7 @@
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -2273,7 +2512,7 @@
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
@@ -2290,11 +2529,11 @@
     </row>
     <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <f>'Northern Trust Master fondsen'!G12</f>
         <v>8.9319673455790307E-4</v>
       </c>
@@ -2306,11 +2545,11 @@
     </row>
     <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <f>SUM(F7:F8)</f>
         <v>9.0901882940875559E-4</v>
       </c>
@@ -2319,7 +2558,7 @@
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -2340,79 +2579,92 @@
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="7" t="s">
-        <v>92</v>
+      <c r="F12" s="3">
+        <f>108396-F5</f>
+        <v>106265</v>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
-      <c r="F13" s="7"/>
+      <c r="F13" s="39">
+        <v>1294</v>
+      </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
-      <c r="F14" s="7"/>
+      <c r="F14" s="4">
+        <f>F12/F6</f>
+        <v>7.889886951317909E-4</v>
+      </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>108</v>
+      </c>
+      <c r="F15" s="4">
+        <f>(F12+F13)/F6</f>
+        <v>7.9859629284976521E-4</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="34">
-        <f>SUM(H7:H10)</f>
-        <v>3.2090188294087553E-3</v>
-      </c>
+      <c r="B17" s="2"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="7">
+      <c r="C18" s="33">
+        <f>SUM(H7:H10)</f>
+        <v>3.2090188294087553E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="32">
         <f>F10+(75%*F9)+0.1%</f>
         <v>3.9817641220565667E-3</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
       <c r="G21" s="5"/>
       <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2422,8 +2674,810 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C5213B5-3E66-4D6C-8B83-264808508A91}">
+  <dimension ref="B2:J24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="32.28515625" customWidth="1"/>
+    <col min="3" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="91.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="J2" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C4" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="13">
+        <v>244</v>
+      </c>
+      <c r="D5" s="13">
+        <v>200</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <v>151</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="J5" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="13">
+        <v>35377446</v>
+      </c>
+      <c r="D6" s="13">
+        <v>337614438</v>
+      </c>
+      <c r="E6" s="13">
+        <v>620074712</v>
+      </c>
+      <c r="F6" s="13">
+        <v>1000756145</v>
+      </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="5">
+        <f>C5/C6</f>
+        <v>6.8970496061247611E-6</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" ref="D7:F7" si="0">D5/D6</f>
+        <v>5.9239172703864047E-7</v>
+      </c>
+      <c r="E7" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" si="0"/>
+        <v>1.5088590837481192E-7</v>
+      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="5">
+        <f>'Northern Trust Master fondsen'!D24</f>
+        <v>1.4240200701548999E-4</v>
+      </c>
+      <c r="D8" s="5">
+        <f>'Northern Trust Master fondsen'!E24</f>
+        <v>1.8879294676940906E-4</v>
+      </c>
+      <c r="E8" s="5">
+        <f>'Northern Trust Master fondsen'!F24</f>
+        <v>5.4497376783190948E-5</v>
+      </c>
+      <c r="F8" s="5">
+        <f>'Northern Trust Master fondsen'!G24</f>
+        <v>4.2326604352244424E-5</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="5">
+        <f>SUM(C7:C8)</f>
+        <v>1.4929905662161474E-4</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" ref="D9:F9" si="1">SUM(D7:D8)</f>
+        <v>1.893853384964477E-4</v>
+      </c>
+      <c r="E9" s="5">
+        <f t="shared" si="1"/>
+        <v>5.4497376783190948E-5</v>
+      </c>
+      <c r="F9" s="5">
+        <f t="shared" si="1"/>
+        <v>4.2477490260619238E-5</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="7">
+        <f>AVERAGE(C9:G9)</f>
+        <v>1.0891481554046815E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1.4E-3</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="F10" s="4">
+        <v>1.4E-3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="7">
+        <f t="shared" ref="H10" si="2">AVERAGE(C10:F10)</f>
+        <v>1.075E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="17">
+        <f>49806-C5</f>
+        <v>49562</v>
+      </c>
+      <c r="D12" s="17">
+        <f>101119-D5</f>
+        <v>100919</v>
+      </c>
+      <c r="E12" s="17">
+        <f>724855-E5</f>
+        <v>724855</v>
+      </c>
+      <c r="F12" s="17">
+        <f>1049269-F5</f>
+        <v>1049118</v>
+      </c>
+      <c r="G12" s="5"/>
+      <c r="H12" s="7"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="17">
+        <v>136</v>
+      </c>
+      <c r="D13" s="17">
+        <v>32602</v>
+      </c>
+      <c r="E13" s="17">
+        <v>1918</v>
+      </c>
+      <c r="F13" s="17">
+        <v>603</v>
+      </c>
+      <c r="G13" s="5"/>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="4">
+        <f>C12/C6</f>
+        <v>1.4009490679457188E-3</v>
+      </c>
+      <c r="D14" s="4">
+        <f t="shared" ref="D14:F14" si="3">D12/D6</f>
+        <v>2.9891790350506276E-4</v>
+      </c>
+      <c r="E14" s="4">
+        <f t="shared" si="3"/>
+        <v>1.1689801018687567E-3</v>
+      </c>
+      <c r="F14" s="4">
+        <f t="shared" si="3"/>
+        <v>1.0483253140554036E-3</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="7">
+        <f>AVERAGE(C14:F14)</f>
+        <v>9.7929309684373551E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="4">
+        <f>(C12+C13)/C6</f>
+        <v>1.4047933251032311E-3</v>
+      </c>
+      <c r="D15" s="4">
+        <f t="shared" ref="D15:F15" si="4">(D12+D13)/D6</f>
+        <v>3.9548367892963156E-4</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" si="4"/>
+        <v>1.1720732775182098E-3</v>
+      </c>
+      <c r="F15" s="4">
+        <f t="shared" si="4"/>
+        <v>1.0489278584444766E-3</v>
+      </c>
+      <c r="G15" s="5"/>
+      <c r="H15" s="7">
+        <f>AVERAGE(C15:F15)</f>
+        <v>1.0053195349988874E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="7">
+        <f>H9+H14</f>
+        <v>1.0882079123842037E-3</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="4">
+        <f>'Tracking Difference'!J21/100</f>
+        <v>3.274999999999998E-3</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="4">
+        <f>C19-C18</f>
+        <v>2.1867920876157943E-3</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="2"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="32">
+        <f>0.15%+AVERAGE(E9:F9)</f>
+        <v>1.5484874335219051E-3</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="32">
+        <f>C22+C20</f>
+        <v>3.7352795211376992E-3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{904897E0-E1C1-4730-BED2-A508F1C09841}">
+  <dimension ref="B2:J24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="32.28515625" customWidth="1"/>
+    <col min="3" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="91.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="J2" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C4" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E4" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="13">
+        <v>739</v>
+      </c>
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13">
+        <v>1729</v>
+      </c>
+      <c r="F5" s="13">
+        <v>331</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="J5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="13">
+        <v>116633513</v>
+      </c>
+      <c r="D6" s="13">
+        <v>256166911</v>
+      </c>
+      <c r="E6" s="13">
+        <v>421319041</v>
+      </c>
+      <c r="F6" s="13">
+        <v>609141396</v>
+      </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="5">
+        <f>C5/C6</f>
+        <v>6.3360862670748841E-6</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" ref="D7:F7" si="0">D5/D6</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
+        <f t="shared" si="0"/>
+        <v>4.1037784475541898E-6</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" si="0"/>
+        <v>5.4338779497428868E-7</v>
+      </c>
+      <c r="G7" s="5"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="4">
+        <f>'Northern Trust Master fondsen'!D18</f>
+        <v>4.0880326741039955E-4</v>
+      </c>
+      <c r="D8" s="4">
+        <f>'Northern Trust Master fondsen'!E18</f>
+        <v>3.2333263888189987E-4</v>
+      </c>
+      <c r="E8" s="4">
+        <f>'Northern Trust Master fondsen'!F18</f>
+        <v>1.4029800153593462E-4</v>
+      </c>
+      <c r="F8" s="4">
+        <f>'Northern Trust Master fondsen'!G18</f>
+        <v>1.0903789686451616E-4</v>
+      </c>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="4">
+        <f>SUM(C7:C8)</f>
+        <v>4.1513935367747443E-4</v>
+      </c>
+      <c r="D9" s="4">
+        <f t="shared" ref="D9:F9" si="1">SUM(D7:D8)</f>
+        <v>3.2333263888189987E-4</v>
+      </c>
+      <c r="E9" s="4">
+        <f t="shared" si="1"/>
+        <v>1.444017799834888E-4</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="1"/>
+        <v>1.0958128465949044E-4</v>
+      </c>
+      <c r="G9" s="5"/>
+      <c r="H9" s="7">
+        <f>AVERAGE(C9:G9)</f>
+        <v>2.4811376430058837E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="4">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="D10" s="4">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="F10" s="4">
+        <v>1.5E-3</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="7">
+        <f t="shared" ref="H10" si="2">AVERAGE(C10:F10)</f>
+        <v>9.2500000000000004E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="17">
+        <f>73959-C5</f>
+        <v>73220</v>
+      </c>
+      <c r="D12" s="17">
+        <f>102247-D5</f>
+        <v>102247</v>
+      </c>
+      <c r="E12" s="17">
+        <f>593572-E5</f>
+        <v>591843</v>
+      </c>
+      <c r="F12" s="17">
+        <f>737120-F5</f>
+        <v>736789</v>
+      </c>
+      <c r="G12" s="5"/>
+      <c r="H12" s="7"/>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="17">
+        <v>85</v>
+      </c>
+      <c r="D13" s="17">
+        <v>868</v>
+      </c>
+      <c r="E13" s="17">
+        <v>2845</v>
+      </c>
+      <c r="F13" s="17">
+        <v>2078</v>
+      </c>
+      <c r="G13" s="5"/>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="4">
+        <f>C12/C6</f>
+        <v>6.2777839847797431E-4</v>
+      </c>
+      <c r="D14" s="4">
+        <f t="shared" ref="D14:F14" si="3">D12/D6</f>
+        <v>3.9914210465691254E-4</v>
+      </c>
+      <c r="E14" s="4">
+        <f t="shared" si="3"/>
+        <v>1.4047383156366769E-3</v>
+      </c>
+      <c r="F14" s="4">
+        <f t="shared" si="3"/>
+        <v>1.2095533234782816E-3</v>
+      </c>
+      <c r="G14" s="5"/>
+      <c r="H14" s="7">
+        <f>AVERAGE(C14:F14)</f>
+        <v>9.1030303556246129E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="4">
+        <f>(C12+C13)/C6</f>
+        <v>6.285071770066636E-4</v>
+      </c>
+      <c r="D15" s="4">
+        <f t="shared" ref="D15:F15" si="4">(D12+D13)/D6</f>
+        <v>4.0253052042306902E-4</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" si="4"/>
+        <v>1.411490918114E-3</v>
+      </c>
+      <c r="F15" s="4">
+        <f t="shared" si="4"/>
+        <v>1.2129646825053406E-3</v>
+      </c>
+      <c r="G15" s="5"/>
+      <c r="H15" s="7">
+        <f>AVERAGE(C15:F15)</f>
+        <v>9.1387332451226834E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="7">
+        <f>H9+H14</f>
+        <v>1.1584167998630497E-3</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="4">
+        <f>'Tracking Difference'!J28/100</f>
+        <v>1.6499999999999959E-3</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="4">
+        <f>C19-C18</f>
+        <v>4.9158320013694616E-4</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="2"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="32">
+        <f>0.15%+AVERAGE(E9:F9)</f>
+        <v>1.6269915323214896E-3</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="32">
+        <f>C22+C20</f>
+        <v>2.1185747324584357E-3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C245834D-4F6D-4A3C-9D7B-51919C891EFD}">
-  <dimension ref="B2:L15"/>
+  <dimension ref="B2:L24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="24.85546875" customWidth="1"/>
@@ -2433,7 +3487,7 @@
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="12"/>
@@ -2441,7 +3495,7 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="I2" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -2479,12 +3533,12 @@
         <v>261252</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="13">
         <v>957946194</v>
@@ -2503,12 +3557,12 @@
         <v>6989496789</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="5">
@@ -2528,7 +3582,7 @@
         <v>4.6130035609743487E-5</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
@@ -2536,12 +3590,12 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
@@ -2566,7 +3620,7 @@
         <v>2019</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J9" s="6"/>
       <c r="L9" s="6"/>
@@ -2575,62 +3629,242 @@
       <c r="B10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="40"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="40">
         <v>63179</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L10" s="4"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3">
+        <v>12</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40">
         <v>0</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="40">
         <v>141467154</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="L11" s="6"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="5">
+        <v>8</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="42">
         <f>G10/AVERAGE(F11:G11)</f>
         <v>8.9319673455790307E-4</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="I13" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B14" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="I14" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2015</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2016</v>
+      </c>
+      <c r="E15" s="1">
+        <v>2017</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2018</v>
+      </c>
+      <c r="G15" s="1">
+        <v>2019</v>
+      </c>
+      <c r="I15" s="9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="I14" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="I15" s="9" t="s">
-        <v>48</v>
-      </c>
       <c r="J15" s="7"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40">
+        <v>45547</v>
+      </c>
+      <c r="E16" s="40">
+        <v>119882</v>
+      </c>
+      <c r="F16" s="40">
+        <v>97972</v>
+      </c>
+      <c r="G16" s="40">
+        <v>119750</v>
+      </c>
+      <c r="I16" s="9"/>
+      <c r="J16" s="7"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="40">
+        <v>25275750</v>
+      </c>
+      <c r="D17" s="40">
+        <v>197555150</v>
+      </c>
+      <c r="E17" s="40">
+        <v>543984587</v>
+      </c>
+      <c r="F17" s="40">
+        <v>852642577</v>
+      </c>
+      <c r="G17" s="40">
+        <v>1343841461</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="5">
+        <f t="shared" ref="D18" si="1">D16/AVERAGE(C17:D17)</f>
+        <v>4.0880326741039955E-4</v>
+      </c>
+      <c r="E18" s="5">
+        <f t="shared" ref="E18" si="2">E16/AVERAGE(D17:E17)</f>
+        <v>3.2333263888189987E-4</v>
+      </c>
+      <c r="F18" s="5">
+        <f t="shared" ref="F18" si="3">F16/AVERAGE(E17:F17)</f>
+        <v>1.4029800153593462E-4</v>
+      </c>
+      <c r="G18" s="5">
+        <f>G16/AVERAGE(F17:G17)</f>
+        <v>1.0903789686451616E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2015</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2016</v>
+      </c>
+      <c r="E21" s="1">
+        <v>2017</v>
+      </c>
+      <c r="F21" s="1">
+        <v>2018</v>
+      </c>
+      <c r="G21" s="1">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="40"/>
+      <c r="D22" s="40">
+        <v>10837</v>
+      </c>
+      <c r="E22" s="40">
+        <v>77254</v>
+      </c>
+      <c r="F22" s="40">
+        <v>45684</v>
+      </c>
+      <c r="G22" s="40">
+        <v>55573</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="40">
+        <v>82931512</v>
+      </c>
+      <c r="D23" s="40">
+        <v>69271399</v>
+      </c>
+      <c r="E23" s="40">
+        <v>749127819</v>
+      </c>
+      <c r="F23" s="40">
+        <v>927429942</v>
+      </c>
+      <c r="G23" s="40">
+        <v>1698483516</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="5">
+        <f t="shared" ref="D24" si="4">D22/AVERAGE(C23:D23)</f>
+        <v>1.4240200701548999E-4</v>
+      </c>
+      <c r="E24" s="5">
+        <f t="shared" ref="E24" si="5">E22/AVERAGE(D23:E23)</f>
+        <v>1.8879294676940906E-4</v>
+      </c>
+      <c r="F24" s="5">
+        <f t="shared" ref="F24" si="6">F22/AVERAGE(E23:F23)</f>
+        <v>5.4497376783190948E-5</v>
+      </c>
+      <c r="G24" s="5">
+        <f>G22/AVERAGE(F23:G23)</f>
+        <v>4.2326604352244424E-5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2639,383 +3873,505 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F528616F-4365-4E03-AA99-F5C2282C78C2}">
-  <dimension ref="B2:P16"/>
+  <dimension ref="B2:N28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="56.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="73" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="19">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="D2" s="19">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="E2" s="19">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="F2" s="19">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="G2" s="19">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="H2" s="19">
-        <v>2017</v>
-      </c>
-      <c r="I2" s="19">
-        <v>2018</v>
-      </c>
-      <c r="J2" s="19">
         <v>2019</v>
       </c>
-      <c r="K2" s="18"/>
-      <c r="L2" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I2" s="18"/>
+      <c r="J2" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="20" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B3" s="20" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="C3" s="21"/>
       <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="E3" s="21">
+        <v>10.55</v>
+      </c>
+      <c r="F3" s="21">
+        <v>8.32</v>
+      </c>
       <c r="G3" s="21">
-        <v>10.55</v>
+        <v>-3.3</v>
       </c>
       <c r="H3" s="21">
-        <v>8.32</v>
-      </c>
-      <c r="I3" s="21">
-        <v>-3.3</v>
-      </c>
-      <c r="J3" s="21">
         <v>30.93</v>
       </c>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="21"/>
-    </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="21"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
+        <v>51</v>
+      </c>
+      <c r="C4" s="21">
+        <v>20.76</v>
+      </c>
+      <c r="D4" s="21">
+        <v>11.13</v>
+      </c>
       <c r="E4" s="21">
-        <v>20.76</v>
+        <v>10.72</v>
       </c>
       <c r="F4" s="21">
-        <v>11.13</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="G4" s="21">
-        <v>10.72</v>
+        <v>-3.12</v>
       </c>
       <c r="H4" s="21">
-        <v>8.5399999999999991</v>
-      </c>
-      <c r="I4" s="21">
-        <v>-3.12</v>
-      </c>
-      <c r="J4" s="21">
         <v>31.17</v>
       </c>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
       <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B5" s="20" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C5" s="21"/>
       <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
+      <c r="E5" s="21">
+        <v>10.07</v>
+      </c>
+      <c r="F5" s="21">
+        <v>7.95</v>
+      </c>
       <c r="G5" s="21">
-        <v>10.07</v>
+        <v>-3.65</v>
       </c>
       <c r="H5" s="21">
-        <v>7.95</v>
-      </c>
-      <c r="I5" s="21">
-        <v>-3.65</v>
-      </c>
-      <c r="J5" s="21">
         <v>30.44</v>
       </c>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="21"/>
-    </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="21"/>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C6" s="21"/>
       <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
+      <c r="E6" s="21">
+        <f>E3-E5</f>
+        <v>0.48000000000000043</v>
+      </c>
+      <c r="F6" s="21">
+        <f>F3-F5</f>
+        <v>0.37000000000000011</v>
+      </c>
       <c r="G6" s="21">
-        <f>G4-G3</f>
-        <v>0.16999999999999993</v>
+        <f>G3-G5</f>
+        <v>0.35000000000000009</v>
       </c>
       <c r="H6" s="21">
-        <f>H4-H3</f>
-        <v>0.21999999999999886</v>
-      </c>
-      <c r="I6" s="21">
-        <f>I4-I3</f>
-        <v>0.17999999999999972</v>
-      </c>
-      <c r="J6" s="21">
-        <f>J4-J3</f>
-        <v>0.24000000000000199</v>
-      </c>
-      <c r="K6" s="18"/>
-      <c r="L6" s="39">
-        <f>AVERAGE(G6:J6)</f>
-        <v>0.20250000000000012</v>
-      </c>
-      <c r="M6" s="21"/>
-      <c r="O6" s="38">
-        <f>AVERAGE(I6:J6)</f>
-        <v>0.21000000000000085</v>
-      </c>
-      <c r="P6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+        <f>H3-H5</f>
+        <v>0.48999999999999844</v>
+      </c>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="21">
+        <f>AVERAGE(E6:H6)</f>
+        <v>0.42249999999999976</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C7" s="21"/>
       <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
+      <c r="E7" s="21">
+        <f>E4-E3</f>
+        <v>0.16999999999999993</v>
+      </c>
+      <c r="F7" s="21">
+        <f>F4-F3</f>
+        <v>0.21999999999999886</v>
+      </c>
       <c r="G7" s="21">
-        <f>G3-G5</f>
-        <v>0.48000000000000043</v>
+        <f>G4-G3</f>
+        <v>0.17999999999999972</v>
       </c>
       <c r="H7" s="21">
-        <f t="shared" ref="H7:J7" si="0">H3-H5</f>
-        <v>0.37000000000000011</v>
-      </c>
-      <c r="I7" s="21">
+        <f>H4-H3</f>
+        <v>0.24000000000000199</v>
+      </c>
+      <c r="I7" s="18"/>
+      <c r="J7" s="38">
+        <f>AVERAGE(E7:H7)</f>
+        <v>0.20250000000000012</v>
+      </c>
+      <c r="K7" s="21"/>
+      <c r="M7" s="36">
+        <f>AVERAGE(G7:H7)</f>
+        <v>0.21000000000000085</v>
+      </c>
+      <c r="N7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B10" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24">
+        <v>12.94</v>
+      </c>
+      <c r="F10" s="24">
+        <v>21.63</v>
+      </c>
+      <c r="G10" s="24">
+        <v>-10.75</v>
+      </c>
+      <c r="H10" s="24">
+        <v>20.82</v>
+      </c>
+      <c r="I10" s="24"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="24"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="24">
+        <v>12.03</v>
+      </c>
+      <c r="D11" s="24">
+        <v>-3.64</v>
+      </c>
+      <c r="E11" s="24">
+        <v>13.57</v>
+      </c>
+      <c r="F11" s="24">
+        <v>21.71</v>
+      </c>
+      <c r="G11" s="24">
+        <v>-10.25</v>
+      </c>
+      <c r="H11" s="24">
+        <v>21.08</v>
+      </c>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="24"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B12" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24">
+        <v>13.14</v>
+      </c>
+      <c r="F12" s="24">
+        <v>21.3</v>
+      </c>
+      <c r="G12" s="24">
+        <v>-10.6</v>
+      </c>
+      <c r="H12" s="24">
+        <v>20.61</v>
+      </c>
+      <c r="I12" s="24"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="24"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B13" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24">
+        <f>E10-E12</f>
+        <v>-0.20000000000000107</v>
+      </c>
+      <c r="F13" s="24">
+        <f>F10-F12</f>
+        <v>0.32999999999999829</v>
+      </c>
+      <c r="G13" s="24">
+        <f>G10-G12</f>
+        <v>-0.15000000000000036</v>
+      </c>
+      <c r="H13" s="24">
+        <f>H10-H12</f>
+        <v>0.21000000000000085</v>
+      </c>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24">
+        <f>AVERAGE(E13:H13)</f>
+        <v>4.7499999999999432E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24">
+        <f>E11-E10</f>
+        <v>0.63000000000000078</v>
+      </c>
+      <c r="F14" s="24">
+        <f>F11-F10</f>
+        <v>8.0000000000001847E-2</v>
+      </c>
+      <c r="G14" s="24">
+        <f>G11-G10</f>
+        <v>0.5</v>
+      </c>
+      <c r="H14" s="24">
+        <f>H11-H10</f>
+        <v>0.25999999999999801</v>
+      </c>
+      <c r="I14" s="24"/>
+      <c r="J14" s="35">
+        <f>AVERAGE(E14:H14)</f>
+        <v>0.36750000000000016</v>
+      </c>
+      <c r="K14" s="24"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17">
+        <v>14.75</v>
+      </c>
+      <c r="F17">
+        <v>7.07</v>
+      </c>
+      <c r="G17">
+        <v>0.35</v>
+      </c>
+      <c r="H17">
+        <v>34.049999999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B18" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18">
+        <v>14.47</v>
+      </c>
+      <c r="F18">
+        <v>6.77</v>
+      </c>
+      <c r="G18">
+        <v>0.02</v>
+      </c>
+      <c r="H18">
+        <v>33.590000000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B19" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19">
+        <v>15.19</v>
+      </c>
+      <c r="F19">
+        <v>7.39</v>
+      </c>
+      <c r="G19">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="H19">
+        <v>34.369999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B20" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20">
+        <f>E17-E18</f>
+        <v>0.27999999999999936</v>
+      </c>
+      <c r="F20">
+        <f t="shared" ref="F20:H20" si="0">F17-F18</f>
+        <v>0.30000000000000071</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="0"/>
-        <v>0.35000000000000009</v>
-      </c>
-      <c r="J7" s="21">
+        <v>0.32999999999999996</v>
+      </c>
+      <c r="H20">
         <f t="shared" si="0"/>
+        <v>0.45999999999999375</v>
+      </c>
+      <c r="K20" s="34">
+        <f>AVERAGE(E20:H20)</f>
+        <v>0.34249999999999847</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B21" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21">
+        <f>E19-E17</f>
+        <v>0.4399999999999995</v>
+      </c>
+      <c r="F21">
+        <f t="shared" ref="F21:H21" si="1">F19-F17</f>
+        <v>0.3199999999999994</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="1"/>
+        <v>0.22999999999999998</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="1"/>
+        <v>0.32000000000000028</v>
+      </c>
+      <c r="J21" s="36">
+        <f>AVERAGE(E21:H21)</f>
+        <v>0.32749999999999979</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B24" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="E24">
+        <v>1.81</v>
+      </c>
+      <c r="F24">
+        <v>10.79</v>
+      </c>
+      <c r="G24">
+        <v>-10.47</v>
+      </c>
+      <c r="H24">
+        <v>26.76</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B25" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25">
+        <v>1.24</v>
+      </c>
+      <c r="F25">
+        <v>10.3</v>
+      </c>
+      <c r="G25">
+        <v>-10.89</v>
+      </c>
+      <c r="H25">
+        <v>26.14</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B26" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26">
+        <v>1.9</v>
+      </c>
+      <c r="F26">
+        <v>10.96</v>
+      </c>
+      <c r="G26">
+        <v>-10.3</v>
+      </c>
+      <c r="H26">
+        <v>26.99</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B27" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="E27">
+        <f>E24-E25</f>
+        <v>0.57000000000000006</v>
+      </c>
+      <c r="F27">
+        <f t="shared" ref="F27:H27" si="2">F24-F25</f>
         <v>0.48999999999999844</v>
       </c>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="21">
-        <f>AVERAGE(G7:J7)</f>
-        <v>0.42249999999999976</v>
-      </c>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B8" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="G8" s="35">
-        <f>G4-G5</f>
-        <v>0.65000000000000036</v>
-      </c>
-      <c r="H8" s="35">
-        <f t="shared" ref="H8:J8" si="1">H4-H5</f>
-        <v>0.58999999999999897</v>
-      </c>
-      <c r="I8" s="35">
-        <f t="shared" si="1"/>
-        <v>0.5299999999999998</v>
-      </c>
-      <c r="J8" s="35">
-        <f t="shared" si="1"/>
-        <v>0.73000000000000043</v>
-      </c>
-      <c r="O8" s="36">
-        <f>AVERAGE(G8:J8)</f>
-        <v>0.62499999999999989</v>
-      </c>
-      <c r="P8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B11" s="22"/>
-      <c r="D11" s="23">
-        <v>2013</v>
-      </c>
-      <c r="E11" s="23">
-        <v>2014</v>
-      </c>
-      <c r="F11" s="23">
-        <v>2015</v>
-      </c>
-      <c r="G11" s="23">
-        <v>2016</v>
-      </c>
-      <c r="H11" s="23">
-        <v>2017</v>
-      </c>
-      <c r="I11" s="23">
-        <v>2018</v>
-      </c>
-      <c r="J11" s="23">
-        <v>2019</v>
-      </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="M11" s="24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B12" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25">
-        <v>12.94</v>
-      </c>
-      <c r="H12" s="25">
-        <v>21.63</v>
-      </c>
-      <c r="I12" s="25">
-        <v>-10.75</v>
-      </c>
-      <c r="J12" s="25">
-        <v>20.82</v>
-      </c>
-      <c r="K12" s="25"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="25"/>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B13" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25">
-        <v>12.03</v>
-      </c>
-      <c r="F13" s="25">
-        <v>-3.64</v>
-      </c>
-      <c r="G13" s="25">
-        <v>13.57</v>
-      </c>
-      <c r="H13" s="25">
-        <v>21.71</v>
-      </c>
-      <c r="I13" s="25">
-        <v>-10.25</v>
-      </c>
-      <c r="J13" s="25">
-        <v>21.08</v>
-      </c>
-      <c r="K13" s="25"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="25"/>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B14" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25">
-        <v>13.14</v>
-      </c>
-      <c r="H14" s="25">
-        <v>21.3</v>
-      </c>
-      <c r="I14" s="25">
-        <v>-10.6</v>
-      </c>
-      <c r="J14" s="25">
-        <v>20.61</v>
-      </c>
-      <c r="K14" s="25"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="25"/>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25">
-        <f>G13-G12</f>
-        <v>0.63000000000000078</v>
-      </c>
-      <c r="H15" s="25">
-        <f>H13-H12</f>
-        <v>8.0000000000001847E-2</v>
-      </c>
-      <c r="I15" s="25">
-        <f>I13-I12</f>
-        <v>0.5</v>
-      </c>
-      <c r="J15" s="25">
-        <f>J13-J12</f>
-        <v>0.25999999999999801</v>
-      </c>
-      <c r="K15" s="25"/>
-      <c r="L15" s="37">
-        <f>AVERAGE(G15:J15)</f>
-        <v>0.36750000000000016</v>
-      </c>
-      <c r="M15" s="25"/>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25">
-        <f>G12-G14</f>
-        <v>-0.20000000000000107</v>
-      </c>
-      <c r="H16" s="25">
-        <f t="shared" ref="H16:J16" si="2">H12-H14</f>
-        <v>0.32999999999999829</v>
-      </c>
-      <c r="I16" s="25">
+      <c r="G27">
         <f t="shared" si="2"/>
-        <v>-0.15000000000000036</v>
-      </c>
-      <c r="J16" s="25">
+        <v>0.41999999999999993</v>
+      </c>
+      <c r="H27">
         <f t="shared" si="2"/>
-        <v>0.21000000000000085</v>
-      </c>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25">
-        <f>AVERAGE(G16:J16)</f>
-        <v>4.7499999999999432E-2</v>
+        <v>0.62000000000000099</v>
+      </c>
+      <c r="K27" s="34">
+        <f>AVERAGE(E27:H27)</f>
+        <v>0.52499999999999991</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B28" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28">
+        <f>E26-E24</f>
+        <v>8.9999999999999858E-2</v>
+      </c>
+      <c r="F28">
+        <f t="shared" ref="F28:H28" si="3">F26-F24</f>
+        <v>0.17000000000000171</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="3"/>
+        <v>0.16999999999999993</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="3"/>
+        <v>0.22999999999999687</v>
+      </c>
+      <c r="J28" s="36">
+        <f>AVERAGE(E28:H28)</f>
+        <v>0.16499999999999959</v>
       </c>
     </row>
   </sheetData>

</xml_diff>